<commit_message>
feat: add pix payment info
</commit_message>
<xml_diff>
--- a/public/bolao_copa2026_final_envio.xlsx
+++ b/public/bolao_copa2026_final_envio.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Palpites 32-avos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regulamento e Pontuação" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Palpites 32-avos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Regulamento e Pontuação" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -122,7 +122,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -144,11 +144,104 @@
         <color rgb="00D3D3D3"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -209,6 +302,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -619,47 +724,33 @@
           <t>🏆 BOLÃO COPA DO MUNDO 2026 — FASE MATA-MATA</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="n"/>
-    </row>
-    <row r="3">
-      <c r="B3" s="1" t="n"/>
-      <c r="C3" s="1" t="n"/>
-      <c r="D3" s="1" t="n"/>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="n"/>
-      <c r="G3" s="1" t="n"/>
-      <c r="H3" s="1" t="n"/>
-    </row>
+    </row>
+    <row r="3"/>
     <row r="5">
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>REGULAMENTO &amp; INSTRUÇÕES:
-1. Preencha seus dados de identificação na Seção 1. Taxa de Inscrição: R$ 50,00.
+1. Preencha seus dados de identificação na Seção 1. Taxa de Inscrição: R$ 50,00. Pagamento via PIX: 71994793104 (Leandro Freire).
 2. Informe o placar final desejado para cada confronto na Seção 2.
 3. IMPORTANTE: Este mesmo palpite valerá para a classificação completa da chave. O pagamento do prêmio ocorrerá somente após o término de todos os jogos desta fase da chave. Não há desempate por estatísticas (prêmio dividido se houver empate).
 4. ENVIO: Após preencher, envie este arquivo para o e-mail: leandroclf@hotmail.com</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
+      <c r="C5" s="23" t="n"/>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="23" t="n"/>
+      <c r="F5" s="23" t="n"/>
+      <c r="G5" s="23" t="n"/>
+      <c r="H5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
+      <c r="B6" s="25" t="n"/>
+      <c r="C6" s="26" t="n"/>
+      <c r="D6" s="26" t="n"/>
+      <c r="E6" s="26" t="n"/>
+      <c r="F6" s="26" t="n"/>
+      <c r="G6" s="26" t="n"/>
+      <c r="H6" s="27" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
@@ -667,12 +758,6 @@
           <t xml:space="preserve"> 1. IDENTIFICAÇÃO DO APOSTADOR (Obrigatório) — Taxa: R$ 50,00</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
@@ -680,12 +765,12 @@
           <t>Nome Completo:</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n"/>
+      <c r="C9" s="28" t="n"/>
       <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="E9" s="29" t="n"/>
+      <c r="F9" s="29" t="n"/>
+      <c r="G9" s="29" t="n"/>
+      <c r="H9" s="30" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
@@ -693,12 +778,12 @@
           <t>Nome de Exibição no Ranking:</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n"/>
+      <c r="C10" s="28" t="n"/>
       <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="E10" s="29" t="n"/>
+      <c r="F10" s="29" t="n"/>
+      <c r="G10" s="29" t="n"/>
+      <c r="H10" s="30" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
@@ -706,12 +791,12 @@
           <t>E-mail de Contato:</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n"/>
+      <c r="C11" s="28" t="n"/>
       <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="E11" s="29" t="n"/>
+      <c r="F11" s="29" t="n"/>
+      <c r="G11" s="29" t="n"/>
+      <c r="H11" s="30" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
@@ -719,12 +804,12 @@
           <t>WhatsApp / Celular:</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n"/>
+      <c r="C12" s="28" t="n"/>
       <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="E12" s="29" t="n"/>
+      <c r="F12" s="29" t="n"/>
+      <c r="G12" s="29" t="n"/>
+      <c r="H12" s="30" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
@@ -732,12 +817,6 @@
           <t xml:space="preserve"> 2. PALPITES — 32-AVOS DE FINAL</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
@@ -1227,9 +1306,9 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="8D2A"/>
   <mergeCells count="12">
-    <mergeCell ref="B8:H8"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B8:H8"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="B10:C10"/>
@@ -1279,25 +1358,14 @@
           <t>📄 REGULAMENTO, PONTUAÇÃO E DIRETRIZES DO BOLÃO</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-    </row>
-    <row r="3">
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-    </row>
+    </row>
+    <row r="3"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>1. CRITÉRIOS DE PONTUAÇÃO POR JOGO</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="15" t="inlineStr">
@@ -1305,7 +1373,6 @@
           <t>Tipo de Acerto / Cenário</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Pontuação</t>
@@ -1323,7 +1390,7 @@
           <t>Placar Exato</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n"/>
+      <c r="C7" s="28" t="n"/>
       <c r="D7" s="18" t="inlineStr">
         <is>
           <t>10 pontos</t>
@@ -1341,7 +1408,7 @@
           <t>Vencedor + 1 Placar Exato (Decisivo)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n"/>
+      <c r="C8" s="28" t="n"/>
       <c r="D8" s="18" t="inlineStr">
         <is>
           <t>5 pontos</t>
@@ -1359,7 +1426,7 @@
           <t>Resultado Correto (Sem Placar Exato)</t>
         </is>
       </c>
-      <c r="C9" s="17" t="n"/>
+      <c r="C9" s="28" t="n"/>
       <c r="D9" s="18" t="inlineStr">
         <is>
           <t>3 pontos</t>
@@ -1377,7 +1444,7 @@
           <t>Invalidez, Ausência ou Erro</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n"/>
+      <c r="C10" s="28" t="n"/>
       <c r="D10" s="18" t="inlineStr">
         <is>
           <t>0 ponto</t>
@@ -1395,9 +1462,6 @@
           <t>2. VALORES, PREMIAÇÃO E DIRETRIZES DE PAGAMENTO</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="19" t="inlineStr">
@@ -1410,8 +1474,6 @@
           <t>O valor da taxa de inscrição será de R$ 50,00 para a classificação completa da fase.</t>
         </is>
       </c>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="19" t="inlineStr">
@@ -1424,8 +1486,6 @@
           <t>Este mesmo palpite preenchido irá valer para a classificação completa desta chave.</t>
         </is>
       </c>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="19" t="inlineStr">
@@ -1438,8 +1498,6 @@
           <t>A PLANILHA PREENCHIDA DEVERÁ SER ENVIADA PARA O E-MAIL: leandroclf@hotmail.com</t>
         </is>
       </c>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="19" t="inlineStr">
@@ -1452,8 +1510,6 @@
           <t>O pagamento da premiação será efetuado apenas APÓS O TÉRMINO DE TODOS OS JOGOS DA CHAVE desta fase.</t>
         </is>
       </c>
-      <c r="D16" s="20" t="n"/>
-      <c r="E16" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="21" t="inlineStr">
@@ -1466,8 +1522,6 @@
           <t>A premiação será definida por fase do bolão e a classificação começa zerada.</t>
         </is>
       </c>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="22" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="19" t="inlineStr">
@@ -1480,8 +1534,6 @@
           <t>APENAS O 1º COLOCADO (CLASSIFICADO) IRÁ RECEBER O PRÊMIO desta fase.</t>
         </is>
       </c>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="19" t="inlineStr">
@@ -1494,8 +1546,6 @@
           <t>NÃO EXISTEM CRITÉRIOS DE DESEMPATE por estatísticas, acertos de placar ou ordem alfabética para a premiação.</t>
         </is>
       </c>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="19" t="inlineStr">
@@ -1508,8 +1558,6 @@
           <t>EM CASO DE EMPATE NA LIDERANÇA, O PRÊMIO SERÁ DIVIDIDO EM PARTES IGUAIS entre todos os líderes empatados.</t>
         </is>
       </c>
-      <c r="D20" s="20" t="n"/>
-      <c r="E20" s="20" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="21" t="inlineStr">
@@ -1522,8 +1570,6 @@
           <t>O pagamento será feito após a conferência final dos resultados e validação da classificação.</t>
         </is>
       </c>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="22" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="21" t="inlineStr">
@@ -1533,11 +1579,9 @@
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
-          <t>O pagamento poderá ser realizado por PIX ou outro meio definido pela organização.</t>
-        </is>
-      </c>
-      <c r="D22" s="22" t="n"/>
-      <c r="E22" s="22" t="n"/>
+          <t>O pagamento será realizado via PIX na chave 71994793104 (Leandro Freire).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="21" t="inlineStr">
@@ -1550,8 +1594,6 @@
           <t>O nome e os dados de pagamento do vencedor deverão ser confirmados antes do repasse.</t>
         </is>
       </c>
-      <c r="D23" s="22" t="n"/>
-      <c r="E23" s="22" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="21" t="inlineStr">
@@ -1564,8 +1606,6 @@
           <t>A organização poderá divulgar o resultado final e o ganhador no site ou em comunicado interno.</t>
         </is>
       </c>
-      <c r="D24" s="22" t="n"/>
-      <c r="E24" s="22" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="21" t="inlineStr">
@@ -1575,11 +1615,9 @@
       </c>
       <c r="C25" s="22" t="inlineStr">
         <is>
-          <t>Caso exista uma taxa administrativa ou retenção para custos do bolão, isso deve ser informado antes do início da fase.</t>
-        </is>
-      </c>
-      <c r="D25" s="22" t="n"/>
-      <c r="E25" s="22" t="n"/>
+          <t>Não existe taxa administrativa nem retenção para custos do bolão.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
@@ -1587,9 +1625,6 @@
           <t>3. CRITÉRIOS DE CLASSIFICAÇÃO GERAL E OPERAÇÃO</t>
         </is>
       </c>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="21" t="inlineStr">
@@ -1602,8 +1637,6 @@
           <t>Maior quantidade de pontos acumulados na fase vigente.</t>
         </is>
       </c>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="22" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="21" t="inlineStr">
@@ -1616,8 +1649,6 @@
           <t>A listagem e ordenação visual no site/tabela pode seguir ordem alfabética em caso de mesma pontuação, mas isso NÃO anula a divisão do prêmio.</t>
         </is>
       </c>
-      <c r="D29" s="22" t="n"/>
-      <c r="E29" s="22" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="21" t="inlineStr">
@@ -1630,8 +1661,6 @@
           <t>Apenas jogos já finalizados e oficialmente apurados entram na soma da tabela.</t>
         </is>
       </c>
-      <c r="D30" s="22" t="n"/>
-      <c r="E30" s="22" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="21" t="inlineStr">
@@ -1644,8 +1673,6 @@
           <t>Palpites ausentes ou inválidos recebem pontuação zero (0).</t>
         </is>
       </c>
-      <c r="D31" s="22" t="n"/>
-      <c r="E31" s="22" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="21" t="inlineStr">
@@ -1658,8 +1685,6 @@
           <t>A classificação geral é recalculada de forma totalmente automática com base nos resultados apurados de toda a chave.</t>
         </is>
       </c>
-      <c r="D32" s="22" t="n"/>
-      <c r="E32" s="22" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>

</xml_diff>

<commit_message>
feat: highlight payment and 90-minute scoring
</commit_message>
<xml_diff>
--- a/public/bolao_copa2026_final_envio.xlsx
+++ b/public/bolao_copa2026_final_envio.xlsx
@@ -241,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -313,6 +313,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -726,13 +738,13 @@
       </c>
     </row>
     <row r="3"/>
-    <row r="5">
-      <c r="B5" s="2" t="inlineStr">
+    <row r="5" ht="24" customHeight="1">
+      <c r="B5" s="31" t="inlineStr">
         <is>
           <t>REGULAMENTO &amp; INSTRUÇÕES:
 1. Preencha seus dados de identificação na Seção 1. Taxa de Inscrição: R$ 50,00. Pagamento via PIX: 71994793104 (Leandro Freire).
 2. Informe o placar final desejado para cada confronto na Seção 2.
-3. IMPORTANTE: Este mesmo palpite valerá para a classificação completa da chave. O pagamento do prêmio ocorrerá somente após o término de todos os jogos desta fase da chave. Não há desempate por estatísticas (prêmio dividido se houver empate).
+3. IMPORTANTE: Este mesmo palpite valerá para a classificação completa da chave. Os resultados serão considerados apenas pelo placar normal da partida, nos 90 minutos, sem prorrogação ou pênaltis. O pagamento do prêmio ocorrerá somente após o término de todos os jogos desta fase da chave. Não há desempate por estatísticas (prêmio dividido se houver empate).
 4. ENVIO: Após preencher, envie este arquivo para o e-mail: leandroclf@hotmail.com</t>
         </is>
       </c>
@@ -743,7 +755,7 @@
       <c r="G5" s="23" t="n"/>
       <c r="H5" s="24" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="24" customHeight="1">
       <c r="B6" s="25" t="n"/>
       <c r="C6" s="26" t="n"/>
       <c r="D6" s="26" t="n"/>
@@ -752,10 +764,10 @@
       <c r="G6" s="26" t="n"/>
       <c r="H6" s="27" t="n"/>
     </row>
-    <row r="8">
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 1. IDENTIFICAÇÃO DO APOSTADOR (Obrigatório) — Taxa: R$ 50,00</t>
+    <row r="8" ht="24" customHeight="1">
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1. IDENTIFICAÇÃO DO APOSTADOR (Obrigatório) — Taxa: R$ 50,00 · PIX 71994793104 (Leandro Freire)</t>
         </is>
       </c>
     </row>
@@ -1307,8 +1319,8 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="8D2A"/>
   <mergeCells count="12">
     <mergeCell ref="D12:H12"/>
+    <mergeCell ref="B8:H8"/>
     <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B8:H8"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="B10:C10"/>
@@ -1511,15 +1523,15 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="30" customHeight="1">
       <c r="B17" s="21" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C17" s="22" t="inlineStr">
-        <is>
-          <t>A premiação será definida por fase do bolão e a classificação começa zerada.</t>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>A premiação será definida por fase do bolão e a classificação começa zerada. Os resultados válidos consideram apenas o placar normal da partida (90 minutos), sem prorrogação ou pênaltis.</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1589,7 @@
           <t>•</t>
         </is>
       </c>
-      <c r="C22" s="22" t="inlineStr">
+      <c r="C22" s="34" t="inlineStr">
         <is>
           <t>O pagamento será realizado via PIX na chave 71994793104 (Leandro Freire).</t>
         </is>
@@ -1613,7 +1625,7 @@
           <t>•</t>
         </is>
       </c>
-      <c r="C25" s="22" t="inlineStr">
+      <c r="C25" s="34" t="inlineStr">
         <is>
           <t>Não existe taxa administrativa nem retenção para custos do bolão.</t>
         </is>

</xml_diff>

<commit_message>
fix: update workbook team names
</commit_message>
<xml_diff>
--- a/public/bolao_copa2026_final_envio.xlsx
+++ b/public/bolao_copa2026_final_envio.xlsx
@@ -472,13 +472,13 @@
         <v>Jogo 73</v>
       </c>
       <c r="C16" t="str">
-        <v>2º Grupo A</v>
+        <v>África do Sul</v>
       </c>
       <c r="E16" t="str">
         <v>x</v>
       </c>
       <c r="F16" t="str">
-        <v>2º Grupo B</v>
+        <v>Canadá</v>
       </c>
       <c r="G16" t="str">
         <v>Canadá</v>
@@ -489,13 +489,13 @@
         <v>Jogo 74</v>
       </c>
       <c r="C17" t="str">
-        <v>1º Grupo E</v>
+        <v>Alemanha</v>
       </c>
       <c r="E17" t="str">
         <v>x</v>
       </c>
       <c r="F17" t="str">
-        <v>Melhor 3º colocado</v>
+        <v>Bósnia</v>
       </c>
       <c r="G17" t="str">
         <v>Bósnia</v>
@@ -506,13 +506,13 @@
         <v>Jogo 75</v>
       </c>
       <c r="C18" t="str">
-        <v>1º Grupo F</v>
+        <v>Holanda</v>
       </c>
       <c r="E18" t="str">
         <v>x</v>
       </c>
       <c r="F18" t="str">
-        <v>2º Grupo C</v>
+        <v>Marrocos</v>
       </c>
       <c r="G18" t="str">
         <v>Marrocos</v>
@@ -523,13 +523,13 @@
         <v>Jogo 76</v>
       </c>
       <c r="C19" t="str">
-        <v>1º Grupo C</v>
+        <v>Brasil</v>
       </c>
       <c r="E19" t="str">
         <v>x</v>
       </c>
       <c r="F19" t="str">
-        <v>2º Grupo F</v>
+        <v>Japão</v>
       </c>
       <c r="G19" t="str">
         <v>Japão</v>
@@ -540,13 +540,13 @@
         <v>Jogo 77</v>
       </c>
       <c r="C20" t="str">
-        <v>1º Grupo I</v>
+        <v>França</v>
       </c>
       <c r="E20" t="str">
         <v>x</v>
       </c>
       <c r="F20" t="str">
-        <v>Melhor 3º colocado</v>
+        <v>Paraguai</v>
       </c>
       <c r="G20" t="str">
         <v>Paraguai</v>
@@ -557,13 +557,13 @@
         <v>Jogo 78</v>
       </c>
       <c r="C21" t="str">
-        <v>2º Grupo E</v>
+        <v>Costa do Marfim</v>
       </c>
       <c r="E21" t="str">
         <v>x</v>
       </c>
       <c r="F21" t="str">
-        <v>2º Grupo I</v>
+        <v>Noruega</v>
       </c>
       <c r="G21" t="str">
         <v>Noruega</v>
@@ -574,13 +574,13 @@
         <v>Jogo 79</v>
       </c>
       <c r="C22" t="str">
-        <v>1º Grupo A</v>
+        <v>México</v>
       </c>
       <c r="E22" t="str">
         <v>x</v>
       </c>
       <c r="F22" t="str">
-        <v>Melhor 3º colocado</v>
+        <v>Equador</v>
       </c>
       <c r="G22" t="str">
         <v>Equador</v>
@@ -591,13 +591,13 @@
         <v>Jogo 80</v>
       </c>
       <c r="C23" t="str">
-        <v>1º Grupo L</v>
+        <v>Inglaterra</v>
       </c>
       <c r="E23" t="str">
         <v>x</v>
       </c>
       <c r="F23" t="str">
-        <v>Melhor 3º colocado</v>
+        <v>Rep. Dem. do Congo</v>
       </c>
       <c r="G23" t="str">
         <v>Rep. Dem. do Congo</v>
@@ -608,13 +608,13 @@
         <v>Jogo 81</v>
       </c>
       <c r="C24" t="str">
-        <v>1º Grupo D</v>
+        <v>Estados Unidos</v>
       </c>
       <c r="E24" t="str">
         <v>x</v>
       </c>
       <c r="F24" t="str">
-        <v>Melhor 3º colocado</v>
+        <v>Suécia</v>
       </c>
       <c r="G24" t="str">
         <v>Suécia</v>
@@ -625,13 +625,13 @@
         <v>Jogo 82</v>
       </c>
       <c r="C25" t="str">
-        <v>1º Grupo G</v>
+        <v>Bélgica</v>
       </c>
       <c r="E25" t="str">
         <v>x</v>
       </c>
       <c r="F25" t="str">
-        <v>Melhor 3º colocado</v>
+        <v>Senegal</v>
       </c>
       <c r="G25" t="str">
         <v>Senegal</v>
@@ -642,13 +642,13 @@
         <v>Jogo 83</v>
       </c>
       <c r="C26" t="str">
-        <v>2º Grupo K</v>
+        <v>Portugal</v>
       </c>
       <c r="E26" t="str">
         <v>x</v>
       </c>
       <c r="F26" t="str">
-        <v>2º Grupo L</v>
+        <v>Croácia</v>
       </c>
       <c r="G26" t="str">
         <v>Croácia</v>
@@ -659,13 +659,13 @@
         <v>Jogo 84</v>
       </c>
       <c r="C27" t="str">
-        <v>1º Grupo H</v>
+        <v>Espanha</v>
       </c>
       <c r="E27" t="str">
         <v>x</v>
       </c>
       <c r="F27" t="str">
-        <v>2º Grupo J</v>
+        <v>Áustria</v>
       </c>
       <c r="G27" t="str">
         <v>Áustria</v>
@@ -676,13 +676,13 @@
         <v>Jogo 85</v>
       </c>
       <c r="C28" t="str">
-        <v>1º Grupo B</v>
+        <v>Suíça</v>
       </c>
       <c r="E28" t="str">
         <v>x</v>
       </c>
       <c r="F28" t="str">
-        <v>Melhor 3º colocado</v>
+        <v>Argélia</v>
       </c>
       <c r="G28" t="str">
         <v>Argélia</v>
@@ -693,13 +693,13 @@
         <v>Jogo 86</v>
       </c>
       <c r="C29" t="str">
-        <v>1º Grupo J</v>
+        <v>Argentina</v>
       </c>
       <c r="E29" t="str">
         <v>x</v>
       </c>
       <c r="F29" t="str">
-        <v>2º Grupo H</v>
+        <v>Cabo Verde</v>
       </c>
       <c r="G29" t="str">
         <v>Cabo Verde</v>
@@ -710,13 +710,13 @@
         <v>Jogo 87</v>
       </c>
       <c r="C30" t="str">
-        <v>1º Grupo K</v>
+        <v>Colômbia</v>
       </c>
       <c r="E30" t="str">
         <v>x</v>
       </c>
       <c r="F30" t="str">
-        <v>Melhor 3º colocado</v>
+        <v>Gana</v>
       </c>
       <c r="G30" t="str">
         <v>Gana</v>
@@ -727,13 +727,13 @@
         <v>Jogo 88</v>
       </c>
       <c r="C31" t="str">
-        <v>2º Grupo D</v>
+        <v>Austrália</v>
       </c>
       <c r="E31" t="str">
         <v>x</v>
       </c>
       <c r="F31" t="str">
-        <v>2º Grupo G</v>
+        <v>Egito</v>
       </c>
       <c r="G31" t="str">
         <v>Egito</v>

</xml_diff>

<commit_message>
Corrige chaveamento e desbloqueio da planilha
</commit_message>
<xml_diff>
--- a/public/bolao_copa2026_final_envio.xlsx
+++ b/public/bolao_copa2026_final_envio.xlsx
@@ -4,9 +4,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Palpites 32-avos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Configurações" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Fontes Oficiais" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Chaveamento Oficial" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Regulamento e Pontuação" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Validação Técnica" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Configurações" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="Regulamento e Pontuação" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -15,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +33,25 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +66,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00103B55"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F1F1A"/>
       </patternFill>
     </fill>
   </fills>
@@ -145,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,6 +180,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -558,20 +595,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>🏆 BOLÃO COPA DO MUNDO 2026 — FASE MATA-MATA</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>VERSÃO DA PLANILHA</t>
-        </is>
-      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>BOLÃO COPA DO MUNDO 2026 — FASE MATA-MATA</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="inlineStr">
         <is>
           <t>2026-06-28 / revisão FIFA</t>
@@ -579,44 +628,32 @@
       </c>
     </row>
     <row r="3">
-      <c r="J3" s="1" t="inlineStr">
-        <is>
-          <t>FONTE OFICIAL</t>
-        </is>
-      </c>
+      <c r="J3" s="1" t="n"/>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 - tabela oficial</t>
+          <t>FIFA oficial</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="J4" s="1" t="inlineStr">
-        <is>
-          <t>DATA DE ATUALIZAÇÃO</t>
-        </is>
-      </c>
+      <c r="J4" s="1" t="n"/>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-28 09:27</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>REGULAMENTO &amp; INSTRUÇÕES:
-1. Preencha seus dados de identificação na Seção 1. Taxa de Inscrição: R$ 50,00. Pagamento via PIX: 71994793104 (Leandro Freire).
-2. Informe o placar final desejado para cada confronto na Seção 2.
-3. IMPORTANTE: Este mesmo palpite valerá para a classificação completa da chave. Os resultados serão considerados apenas pelo placar normal da partida, nos 90 minutos, sem prorrogação ou pênaltis.
-4. ENVIO: Após preencher, envie este arquivo para o e-mail: leandroclf@hotmail.com</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="inlineStr">
-        <is>
-          <t>REFERÊNCIA</t>
-        </is>
-      </c>
+1. Preencha os dados de identificação.
+2. Informe os palpites dos 32 avos.
+3. Resultados válidos: apenas 90 minutos.
+4. Prorrogação e pênaltis servem apenas para definir classificado.</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="n"/>
       <c r="K5" s="1" t="inlineStr">
         <is>
           <t>48 seleções · 12 grupos · 32 avos</t>
@@ -624,102 +661,88 @@
       </c>
     </row>
     <row r="6"/>
-    <row r="7">
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>DADOS DO APOSTADOR</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
-      <c r="B8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 1. IDENTIFICAÇÃO DO APOSTADOR (Obrigatório) — Taxa: R$ 50,00 · PIX 71994793104 (Leandro Freire)</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>1. IDENTIFICAÇÃO DO APOSTADOR (Obrigatório) — Taxa: R$ 50,00 · PIX 71994793104 (Leandro Freire)</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr">
         <is>
           <t>ID ÚNICO</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>BOLAO-2026-CC3F032E</t>
-        </is>
-      </c>
+      <c r="K8" s="1" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Nome Completo:</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>DATA/HORA ENVIO</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="C9" s="13" t="inlineStr"/>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>DATA/HORA DO ENVIO</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Nome de Exibição no Ranking:</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr"/>
+      <c r="J10" s="1" t="inlineStr">
         <is>
           <t>STATUS PAGAMENTO</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>E-mail de Contato:</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr"/>
+      <c r="J11" s="1" t="inlineStr">
         <is>
           <t>CONFIRMAÇÃO PIX</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K11" s="13" t="inlineStr">
         <is>
           <t>Não confirmado</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>WhatsApp / Celular:</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr"/>
+      <c r="J12" s="1" t="inlineStr">
         <is>
           <t>VALOR INSCRIÇÃO</t>
         </is>
       </c>
-      <c r="K12" s="3" t="n">
+      <c r="K12" s="13" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 2. PALPITES — 32-AVOS DE FINAL</t>
-        </is>
-      </c>
-    </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -753,7 +776,37 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Status do Jogo</t>
+          <t>Classificado</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Decisão</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>ET M</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>ET V</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Pen M</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Pen V</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -765,26 +818,27 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>África do Sul</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="n"/>
+          <t>2º Grupo A</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="n"/>
       <c r="E16" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>Canadá</t>
-        </is>
-      </c>
+      <c r="F16" s="13" t="n"/>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>Canadá</t>
-        </is>
-      </c>
-      <c r="H16" s="1" t="inlineStr">
+          <t>2º Grupo B</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="13" t="n"/>
+      <c r="K16" s="13" t="n"/>
+      <c r="L16" s="13" t="n"/>
+      <c r="M16" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -798,26 +852,27 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>Alemanha</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="n"/>
+          <t>1º Grupo E</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="n"/>
       <c r="E17" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>Bósnia</t>
-        </is>
-      </c>
+      <c r="F17" s="13" t="n"/>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>Bósnia</t>
-        </is>
-      </c>
-      <c r="H17" s="1" t="inlineStr">
+          <t>Melhor 3º colocado: Grupos A/B/C/D/F</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="n"/>
+      <c r="J17" s="13" t="n"/>
+      <c r="K17" s="13" t="n"/>
+      <c r="L17" s="13" t="n"/>
+      <c r="M17" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -831,26 +886,27 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>Holanda</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="n"/>
+          <t>1º Grupo F</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n"/>
       <c r="E18" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
-        <is>
-          <t>Marrocos</t>
-        </is>
-      </c>
+      <c r="F18" s="13" t="n"/>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>Marrocos</t>
-        </is>
-      </c>
-      <c r="H18" s="1" t="inlineStr">
+          <t>2º Grupo C</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="13" t="n"/>
+      <c r="K18" s="13" t="n"/>
+      <c r="L18" s="13" t="n"/>
+      <c r="M18" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -864,26 +920,27 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="n"/>
+          <t>1º Grupo C</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n"/>
       <c r="E19" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
-        <is>
-          <t>Japão</t>
-        </is>
-      </c>
+      <c r="F19" s="13" t="n"/>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>Japão</t>
-        </is>
-      </c>
-      <c r="H19" s="1" t="inlineStr">
+          <t>2º Grupo F</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="13" t="n"/>
+      <c r="M19" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -897,26 +954,27 @@
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>França</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="n"/>
+          <t>1º Grupo I</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n"/>
       <c r="E20" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>Paraguai</t>
-        </is>
-      </c>
+      <c r="F20" s="13" t="n"/>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>Paraguai</t>
-        </is>
-      </c>
-      <c r="H20" s="1" t="inlineStr">
+          <t>Melhor 3º colocado: Grupos C/D/F/G/H</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="n"/>
+      <c r="J20" s="13" t="n"/>
+      <c r="K20" s="13" t="n"/>
+      <c r="L20" s="13" t="n"/>
+      <c r="M20" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -930,26 +988,27 @@
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>Costa do Marfim</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="n"/>
+          <t>2º Grupo E</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="n"/>
       <c r="E21" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
-        <is>
-          <t>Noruega</t>
-        </is>
-      </c>
+      <c r="F21" s="13" t="n"/>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>Noruega</t>
-        </is>
-      </c>
-      <c r="H21" s="1" t="inlineStr">
+          <t>2º Grupo I</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="n"/>
+      <c r="K21" s="13" t="n"/>
+      <c r="L21" s="13" t="n"/>
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -963,26 +1022,27 @@
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D22" s="1" t="n"/>
+          <t>1º Grupo A</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n"/>
       <c r="E22" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
-        <is>
-          <t>Equador</t>
-        </is>
-      </c>
+      <c r="F22" s="13" t="n"/>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>Equador</t>
-        </is>
-      </c>
-      <c r="H22" s="1" t="inlineStr">
+          <t>Melhor 3º colocado: Grupos C/E/F/H/I</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="n"/>
+      <c r="I22" s="13" t="n"/>
+      <c r="J22" s="13" t="n"/>
+      <c r="K22" s="13" t="n"/>
+      <c r="L22" s="13" t="n"/>
+      <c r="M22" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -996,26 +1056,27 @@
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>Inglaterra</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="n"/>
+          <t>1º Grupo L</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n"/>
       <c r="E23" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
-        <is>
-          <t>Rep. Dem. do Congo</t>
-        </is>
-      </c>
+      <c r="F23" s="13" t="n"/>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>Rep. Dem. do Congo</t>
-        </is>
-      </c>
-      <c r="H23" s="1" t="inlineStr">
+          <t>Melhor 3º colocado: Grupos E/H/I/J/K</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="13" t="n"/>
+      <c r="K23" s="13" t="n"/>
+      <c r="L23" s="13" t="n"/>
+      <c r="M23" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1029,26 +1090,27 @@
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="n"/>
+          <t>1º Grupo D</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n"/>
       <c r="E24" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
-        <is>
-          <t>Suécia</t>
-        </is>
-      </c>
+      <c r="F24" s="13" t="n"/>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>Suécia</t>
-        </is>
-      </c>
-      <c r="H24" s="1" t="inlineStr">
+          <t>Melhor 3º colocado: Grupos B/E/F/I/J</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="n"/>
+      <c r="J24" s="13" t="n"/>
+      <c r="K24" s="13" t="n"/>
+      <c r="L24" s="13" t="n"/>
+      <c r="M24" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1062,26 +1124,27 @@
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>Bélgica</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="n"/>
+          <t>1º Grupo G</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n"/>
       <c r="E25" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
+      <c r="F25" s="13" t="n"/>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-      <c r="H25" s="1" t="inlineStr">
+          <t>Melhor 3º colocado: Grupos A/E/H/I/J</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
+      <c r="K25" s="13" t="n"/>
+      <c r="L25" s="13" t="n"/>
+      <c r="M25" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1095,26 +1158,27 @@
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="n"/>
+          <t>2º Grupo K</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n"/>
       <c r="E26" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
-        <is>
-          <t>Croácia</t>
-        </is>
-      </c>
+      <c r="F26" s="13" t="n"/>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>Croácia</t>
-        </is>
-      </c>
-      <c r="H26" s="1" t="inlineStr">
+          <t>2º Grupo L</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
+      <c r="K26" s="13" t="n"/>
+      <c r="L26" s="13" t="n"/>
+      <c r="M26" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1128,26 +1192,27 @@
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>Espanha</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="n"/>
+          <t>1º Grupo H</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n"/>
       <c r="E27" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
-        <is>
-          <t>Áustria</t>
-        </is>
-      </c>
+      <c r="F27" s="13" t="n"/>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>Áustria</t>
-        </is>
-      </c>
-      <c r="H27" s="1" t="inlineStr">
+          <t>2º Grupo J</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="13" t="n"/>
+      <c r="L27" s="13" t="n"/>
+      <c r="M27" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1161,26 +1226,27 @@
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>Suíça</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="n"/>
+          <t>1º Grupo B</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="n"/>
       <c r="E28" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
-        <is>
-          <t>Argélia</t>
-        </is>
-      </c>
+      <c r="F28" s="13" t="n"/>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>Argélia</t>
-        </is>
-      </c>
-      <c r="H28" s="1" t="inlineStr">
+          <t>Melhor 3º colocado: Grupos E/F/G/I/J</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="13" t="n"/>
+      <c r="L28" s="13" t="n"/>
+      <c r="M28" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1194,26 +1260,27 @@
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="D29" s="1" t="n"/>
+          <t>1º Grupo J</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="n"/>
       <c r="E29" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
-        <is>
-          <t>Cabo Verde</t>
-        </is>
-      </c>
+      <c r="F29" s="13" t="n"/>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>Cabo Verde</t>
-        </is>
-      </c>
-      <c r="H29" s="1" t="inlineStr">
+          <t>2º Grupo H</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
+      <c r="K29" s="13" t="n"/>
+      <c r="L29" s="13" t="n"/>
+      <c r="M29" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1227,26 +1294,27 @@
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>Colômbia</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="n"/>
+          <t>1º Grupo K</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="n"/>
       <c r="E30" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
-        <is>
-          <t>Gana</t>
-        </is>
-      </c>
+      <c r="F30" s="13" t="n"/>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>Gana</t>
-        </is>
-      </c>
-      <c r="H30" s="1" t="inlineStr">
+          <t>Melhor 3º colocado: Grupos D/E/I/J/L</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="n"/>
+      <c r="J30" s="13" t="n"/>
+      <c r="K30" s="13" t="n"/>
+      <c r="L30" s="13" t="n"/>
+      <c r="M30" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1260,26 +1328,27 @@
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>Austrália</t>
-        </is>
-      </c>
-      <c r="D31" s="1" t="n"/>
+          <t>2º Grupo D</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="n"/>
       <c r="E31" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
-        <is>
-          <t>Egito</t>
-        </is>
-      </c>
+      <c r="F31" s="13" t="n"/>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>Egito</t>
-        </is>
-      </c>
-      <c r="H31" s="1" t="inlineStr">
+          <t>2º Grupo G</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="n"/>
+      <c r="J31" s="13" t="n"/>
+      <c r="K31" s="13" t="n"/>
+      <c r="L31" s="13" t="n"/>
+      <c r="M31" s="1" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
@@ -1287,33 +1356,38 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="8D2A"/>
-  <mergeCells count="12">
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D11:H11"/>
+  <mergeCells count="2">
+    <mergeCell ref="B5:H6"/>
     <mergeCell ref="B2:H3"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B5:H6"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="B12:C12"/>
   </mergeCells>
-  <dataValidations count="4">
-    <dataValidation sqref="D16:D31 F16:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+  <dataValidations count="8">
+    <dataValidation sqref="D16:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Apenas números inteiros entre 0 e 20 são permitidos." prompt="Informe um inteiro entre 0 e 20." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation sqref="F16:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Apenas números inteiros entre 0 e 20 são permitidos." prompt="Informe um inteiro entre 0 e 20." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation sqref="J16:J31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Apenas números inteiros entre 0 e 20 são permitidos." prompt="Informe um inteiro entre 0 e 20." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation sqref="K16:K31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Apenas números inteiros entre 0 e 20 são permitidos." prompt="Informe um inteiro entre 0 e 20." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>20</formula2>
     </dataValidation>
     <dataValidation sqref="H16:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Pendente,Programado,Em andamento,Finalizado"</formula1>
+      <formula1>"Mandante,Visitante"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I16:I31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Tempo normal,Prorrogação,Pênaltis"</formula1>
     </dataValidation>
     <dataValidation sqref="K10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Pendente,Confirmado,Isento,Cancelado"</formula1>
+      <formula1>"Pendente,Confirmado"</formula1>
     </dataValidation>
     <dataValidation sqref="K11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Não confirmado,Confirmado"</formula1>
+      <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1326,149 +1400,97 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Parâmetro</t>
+          <t>Fonte</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Valor</t>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Uso</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>versao_planilha</t>
+          <t>Formato da competição</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28 / revisão FIFA</t>
+          <t>https://www.fifa.com/pt/tournaments/mens/worldcup/canadamexicousa2026/articles/copa-mundo-2026-tabela-jogos</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>48 seleções, 12 grupos e classificação ao mata-mata</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>fonte_oficial</t>
+          <t>Calendário/jogos</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
           <t>https://www.fifa.com/pt/tournaments/mens/worldcup/canadamexicousa2026/articles/copa-mundo-2026-tabela-jogos</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Jogos, datas e estádios publicados pela FIFA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>referencia_formato</t>
+          <t>Chaveamento mata-mata</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>48 seleções · 12 grupos · 32 avos · 8 melhores terceiros</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>taxa_inscricao</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>50</v>
+          <t>https://www.fifa.com/pt/tournaments/mens/worldcup/canadamexicousa2026/articles/tabela-copa-mundo-2026-fase-final-mata-mata</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Chaveamento oficial da fase eliminatória</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>sem_taxa_administrativa</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>status_pagamento_list</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Pendente,Confirmado,Isento,Cancelado</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>status_jogo_list</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Pendente,Programado,Em andamento,Finalizado</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>decisao_list</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Tempo normal,Prorrogação,Pênaltis</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>classificado_list</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Mandante,Visitante</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>placar_min</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>placar_max</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>20</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Última conferência</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-28 09:27</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Validação manual</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1494,10 +1516,10 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -1514,12 +1536,12 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Mandante</t>
+          <t>Mandante (oficial)</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Visitante</t>
+          <t>Visitante (oficial)</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -1581,12 +1603,12 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>África do Sul</t>
+          <t>2º Grupo A</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Canadá</t>
+          <t>2º Grupo B</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -1597,16 +1619,20 @@
       <c r="F2" s="1" t="inlineStr"/>
       <c r="G2" s="1" t="inlineStr"/>
       <c r="H2" s="1" t="inlineStr"/>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1">
+      <c r="I2" s="13" t="n"/>
+      <c r="J2" s="13" t="n"/>
+      <c r="K2" s="13">
         <f>IF(OR(I2="",J2=""),"",IF(I2&gt;J2,C2,IF(J2&gt;I2,D2,"")))</f>
         <v/>
       </c>
-      <c r="L2" s="1" t="inlineStr"/>
+      <c r="L2" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M2" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1623,12 +1649,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Alemanha</t>
+          <t>1º Grupo E</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Bósnia</t>
+          <t>Melhor 3º colocado: Grupos A/B/C/D/F</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -1639,16 +1665,20 @@
       <c r="F3" s="1" t="inlineStr"/>
       <c r="G3" s="1" t="inlineStr"/>
       <c r="H3" s="1" t="inlineStr"/>
-      <c r="I3" s="1" t="n"/>
-      <c r="J3" s="1" t="n"/>
-      <c r="K3" s="1">
+      <c r="I3" s="13" t="n"/>
+      <c r="J3" s="13" t="n"/>
+      <c r="K3" s="13">
         <f>IF(OR(I3="",J3=""),"",IF(I3&gt;J3,C3,IF(J3&gt;I3,D3,"")))</f>
         <v/>
       </c>
-      <c r="L3" s="1" t="inlineStr"/>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M3" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1665,12 +1695,12 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>Holanda</t>
+          <t>1º Grupo F</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>Marrocos</t>
+          <t>2º Grupo C</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
@@ -1681,16 +1711,20 @@
       <c r="F4" s="1" t="inlineStr"/>
       <c r="G4" s="1" t="inlineStr"/>
       <c r="H4" s="1" t="inlineStr"/>
-      <c r="I4" s="1" t="n"/>
-      <c r="J4" s="1" t="n"/>
-      <c r="K4" s="1">
+      <c r="I4" s="13" t="n"/>
+      <c r="J4" s="13" t="n"/>
+      <c r="K4" s="13">
         <f>IF(OR(I4="",J4=""),"",IF(I4&gt;J4,C4,IF(J4&gt;I4,D4,"")))</f>
         <v/>
       </c>
-      <c r="L4" s="1" t="inlineStr"/>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M4" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1707,12 +1741,12 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>1º Grupo C</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Japão</t>
+          <t>2º Grupo F</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -1723,16 +1757,20 @@
       <c r="F5" s="1" t="inlineStr"/>
       <c r="G5" s="1" t="inlineStr"/>
       <c r="H5" s="1" t="inlineStr"/>
-      <c r="I5" s="1" t="n"/>
-      <c r="J5" s="1" t="n"/>
-      <c r="K5" s="1">
+      <c r="I5" s="13" t="n"/>
+      <c r="J5" s="13" t="n"/>
+      <c r="K5" s="13">
         <f>IF(OR(I5="",J5=""),"",IF(I5&gt;J5,C5,IF(J5&gt;I5,D5,"")))</f>
         <v/>
       </c>
-      <c r="L5" s="1" t="inlineStr"/>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M5" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1749,12 +1787,12 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>França</t>
+          <t>1º Grupo I</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Paraguai</t>
+          <t>Melhor 3º colocado: Grupos C/D/F/G/H</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -1765,16 +1803,20 @@
       <c r="F6" s="1" t="inlineStr"/>
       <c r="G6" s="1" t="inlineStr"/>
       <c r="H6" s="1" t="inlineStr"/>
-      <c r="I6" s="1" t="n"/>
-      <c r="J6" s="1" t="n"/>
-      <c r="K6" s="1">
+      <c r="I6" s="13" t="n"/>
+      <c r="J6" s="13" t="n"/>
+      <c r="K6" s="13">
         <f>IF(OR(I6="",J6=""),"",IF(I6&gt;J6,C6,IF(J6&gt;I6,D6,"")))</f>
         <v/>
       </c>
-      <c r="L6" s="1" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M6" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1791,12 +1833,12 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>Costa do Marfim</t>
+          <t>2º Grupo E</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>2º Grupo I</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -1807,16 +1849,20 @@
       <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="1" t="inlineStr"/>
       <c r="H7" s="1" t="inlineStr"/>
-      <c r="I7" s="1" t="n"/>
-      <c r="J7" s="1" t="n"/>
-      <c r="K7" s="1">
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="13" t="n"/>
+      <c r="K7" s="13">
         <f>IF(OR(I7="",J7=""),"",IF(I7&gt;J7,C7,IF(J7&gt;I7,D7,"")))</f>
         <v/>
       </c>
-      <c r="L7" s="1" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M7" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1833,12 +1879,12 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>1º Grupo A</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>Equador</t>
+          <t>Melhor 3º colocado: Grupos C/E/F/H/I</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
@@ -1849,16 +1895,20 @@
       <c r="F8" s="1" t="inlineStr"/>
       <c r="G8" s="1" t="inlineStr"/>
       <c r="H8" s="1" t="inlineStr"/>
-      <c r="I8" s="1" t="n"/>
-      <c r="J8" s="1" t="n"/>
-      <c r="K8" s="1">
+      <c r="I8" s="13" t="n"/>
+      <c r="J8" s="13" t="n"/>
+      <c r="K8" s="13">
         <f>IF(OR(I8="",J8=""),"",IF(I8&gt;J8,C8,IF(J8&gt;I8,D8,"")))</f>
         <v/>
       </c>
-      <c r="L8" s="1" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M8" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1875,12 +1925,12 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>Inglaterra</t>
+          <t>1º Grupo L</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>Rep. Dem. do Congo</t>
+          <t>Melhor 3º colocado: Grupos E/H/I/J/K</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -1891,16 +1941,20 @@
       <c r="F9" s="1" t="inlineStr"/>
       <c r="G9" s="1" t="inlineStr"/>
       <c r="H9" s="1" t="inlineStr"/>
-      <c r="I9" s="1" t="n"/>
-      <c r="J9" s="1" t="n"/>
-      <c r="K9" s="1">
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13" t="n"/>
+      <c r="K9" s="13">
         <f>IF(OR(I9="",J9=""),"",IF(I9&gt;J9,C9,IF(J9&gt;I9,D9,"")))</f>
         <v/>
       </c>
-      <c r="L9" s="1" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M9" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1917,12 +1971,12 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>1º Grupo D</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Suécia</t>
+          <t>Melhor 3º colocado: Grupos B/E/F/I/J</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
@@ -1933,16 +1987,20 @@
       <c r="F10" s="1" t="inlineStr"/>
       <c r="G10" s="1" t="inlineStr"/>
       <c r="H10" s="1" t="inlineStr"/>
-      <c r="I10" s="1" t="n"/>
-      <c r="J10" s="1" t="n"/>
-      <c r="K10" s="1">
+      <c r="I10" s="13" t="n"/>
+      <c r="J10" s="13" t="n"/>
+      <c r="K10" s="13">
         <f>IF(OR(I10="",J10=""),"",IF(I10&gt;J10,C10,IF(J10&gt;I10,D10,"")))</f>
         <v/>
       </c>
-      <c r="L10" s="1" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M10" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -1959,12 +2017,12 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>Bélgica</t>
+          <t>1º Grupo G</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Melhor 3º colocado: Grupos A/E/H/I/J</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
@@ -1975,16 +2033,20 @@
       <c r="F11" s="1" t="inlineStr"/>
       <c r="G11" s="1" t="inlineStr"/>
       <c r="H11" s="1" t="inlineStr"/>
-      <c r="I11" s="1" t="n"/>
-      <c r="J11" s="1" t="n"/>
-      <c r="K11" s="1">
+      <c r="I11" s="13" t="n"/>
+      <c r="J11" s="13" t="n"/>
+      <c r="K11" s="13">
         <f>IF(OR(I11="",J11=""),"",IF(I11&gt;J11,C11,IF(J11&gt;I11,D11,"")))</f>
         <v/>
       </c>
-      <c r="L11" s="1" t="inlineStr"/>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M11" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -2001,12 +2063,12 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>2º Grupo K</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>Croácia</t>
+          <t>2º Grupo L</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
@@ -2017,16 +2079,20 @@
       <c r="F12" s="1" t="inlineStr"/>
       <c r="G12" s="1" t="inlineStr"/>
       <c r="H12" s="1" t="inlineStr"/>
-      <c r="I12" s="1" t="n"/>
-      <c r="J12" s="1" t="n"/>
-      <c r="K12" s="1">
+      <c r="I12" s="13" t="n"/>
+      <c r="J12" s="13" t="n"/>
+      <c r="K12" s="13">
         <f>IF(OR(I12="",J12=""),"",IF(I12&gt;J12,C12,IF(J12&gt;I12,D12,"")))</f>
         <v/>
       </c>
-      <c r="L12" s="1" t="inlineStr"/>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M12" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -2043,12 +2109,12 @@
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>Espanha</t>
+          <t>1º Grupo H</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>Áustria</t>
+          <t>2º Grupo J</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -2059,16 +2125,20 @@
       <c r="F13" s="1" t="inlineStr"/>
       <c r="G13" s="1" t="inlineStr"/>
       <c r="H13" s="1" t="inlineStr"/>
-      <c r="I13" s="1" t="n"/>
-      <c r="J13" s="1" t="n"/>
-      <c r="K13" s="1">
+      <c r="I13" s="13" t="n"/>
+      <c r="J13" s="13" t="n"/>
+      <c r="K13" s="13">
         <f>IF(OR(I13="",J13=""),"",IF(I13&gt;J13,C13,IF(J13&gt;I13,D13,"")))</f>
         <v/>
       </c>
-      <c r="L13" s="1" t="inlineStr"/>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M13" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -2085,12 +2155,12 @@
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>Suíça</t>
+          <t>1º Grupo B</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>Argélia</t>
+          <t>Melhor 3º colocado: Grupos E/F/G/I/J</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
@@ -2101,16 +2171,20 @@
       <c r="F14" s="1" t="inlineStr"/>
       <c r="G14" s="1" t="inlineStr"/>
       <c r="H14" s="1" t="inlineStr"/>
-      <c r="I14" s="1" t="n"/>
-      <c r="J14" s="1" t="n"/>
-      <c r="K14" s="1">
+      <c r="I14" s="13" t="n"/>
+      <c r="J14" s="13" t="n"/>
+      <c r="K14" s="13">
         <f>IF(OR(I14="",J14=""),"",IF(I14&gt;J14,C14,IF(J14&gt;I14,D14,"")))</f>
         <v/>
       </c>
-      <c r="L14" s="1" t="inlineStr"/>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M14" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -2127,12 +2201,12 @@
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>1º Grupo J</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>Cabo Verde</t>
+          <t>2º Grupo H</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -2143,16 +2217,20 @@
       <c r="F15" s="1" t="inlineStr"/>
       <c r="G15" s="1" t="inlineStr"/>
       <c r="H15" s="1" t="inlineStr"/>
-      <c r="I15" s="1" t="n"/>
-      <c r="J15" s="1" t="n"/>
-      <c r="K15" s="1">
+      <c r="I15" s="13" t="n"/>
+      <c r="J15" s="13" t="n"/>
+      <c r="K15" s="13">
         <f>IF(OR(I15="",J15=""),"",IF(I15&gt;J15,C15,IF(J15&gt;I15,D15,"")))</f>
         <v/>
       </c>
-      <c r="L15" s="1" t="inlineStr"/>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M15" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -2169,12 +2247,12 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>Colômbia</t>
+          <t>1º Grupo K</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>Gana</t>
+          <t>Melhor 3º colocado: Grupos D/E/I/J/L</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
@@ -2185,16 +2263,20 @@
       <c r="F16" s="1" t="inlineStr"/>
       <c r="G16" s="1" t="inlineStr"/>
       <c r="H16" s="1" t="inlineStr"/>
-      <c r="I16" s="1" t="n"/>
-      <c r="J16" s="1" t="n"/>
-      <c r="K16" s="1">
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="13" t="n"/>
+      <c r="K16" s="13">
         <f>IF(OR(I16="",J16=""),"",IF(I16&gt;J16,C16,IF(J16&gt;I16,D16,"")))</f>
         <v/>
       </c>
-      <c r="L16" s="1" t="inlineStr"/>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M16" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
         </is>
       </c>
     </row>
@@ -2211,12 +2293,12 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>Austrália</t>
+          <t>2º Grupo D</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>Egito</t>
+          <t>2º Grupo G</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -2227,16 +2309,169 @@
       <c r="F17" s="1" t="inlineStr"/>
       <c r="G17" s="1" t="inlineStr"/>
       <c r="H17" s="1" t="inlineStr"/>
-      <c r="I17" s="1" t="n"/>
-      <c r="J17" s="1" t="n"/>
-      <c r="K17" s="1">
+      <c r="I17" s="13" t="n"/>
+      <c r="J17" s="13" t="n"/>
+      <c r="K17" s="13">
         <f>IF(OR(I17="",J17=""),"",IF(I17&gt;J17,C17,IF(J17&gt;I17,D17,"")))</f>
         <v/>
       </c>
-      <c r="L17" s="1" t="inlineStr"/>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>Tempo normal</t>
+        </is>
+      </c>
       <c r="M17" s="1" t="inlineStr">
         <is>
-          <t>FIFA World Cup 2026 official bracket</t>
+          <t>FIFA official bracket</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="8D2A"/>
+  <dataValidations count="2">
+    <dataValidation sqref="I2:I17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation sqref="J2:J17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Detalhe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Confrontos corrigidos</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>R32 reescrito com nomenclatura oficial FIFA. Sem seleções fixas fora dos slots oficiais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Input desbloqueado</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Nome, e-mail, WhatsApp, placares, classificado, decisão, prorrogação e pênaltis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Protegido</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cabeçalhos, fórmulas, estrutura, nomes das fases e células de cálculo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Validações</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Inteiros 0-20; listas suspensas para status, decisão e confirmação PIX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Divergências anteriores</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Havia seleções fixas e palpites bloqueados na linha de 32 avos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Simulação de uso</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Apostador consegue digitar dados e palpites sem destravar fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fontes oficiais</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>URLs FIFA registradas em aba própria e data/hora da última conferência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Os confrontos foram mantidos como slots oficiais porque a classificação final de grupo ainda é variável.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Última conferência</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-28 09:27</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2481,176 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Parâmetro</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>versao_planilha</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-28 / revisão FIFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>fonte_formato</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fifa.com/pt/tournaments/mens/worldcup/canadamexicousa2026/articles/copa-mundo-2026-tabela-jogos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>fonte_calendario</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fifa.com/pt/tournaments/mens/worldcup/canadamexicousa2026/articles/copa-mundo-2026-tabela-jogos</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>fonte_chaveamento</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fifa.com/pt/tournaments/mens/worldcup/canadamexicousa2026/articles/tabela-copa-mundo-2026-fase-final-mata-mata</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>taxa_inscricao</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>sem_taxa_administrativa</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>status_pagamento_list</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Pendente,Confirmado,Isento,Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>status_jogo_list</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Pendente,Programado,Em andamento,Finalizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>decisao_list</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Tempo normal,Prorrogação,Pênaltis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>classificado_list</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Mandante,Visitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>placar_min</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>placar_max</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="8D2A"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2278,183 +2682,183 @@
       <c r="E3" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>1. REFERÊNCIA OFICIAL E FORMATO</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>A competição segue a Copa do Mundo FIFA 2026 com 48 seleções, 12 grupos, classificação dos 2 primeiros e dos 8 melhores terceiros, e mata-mata iniciando nos 32 avos de final.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Fonte oficial: FIFA (tabela de jogos e chaveamento oficial).</t>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Fonte oficial: FIFA.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>2. PONTUAÇÃO</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Pontuação</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Critério</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>10 pontos</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Placar exato.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>5 pontos</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Vencedor correto + um placar exato em jogos decisivos.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>3 pontos</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Resultado correto (vitória ou empate) sem placar exato.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>0 ponto</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Resultado incorreto, ausência de palpite ou jogo não apurado.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>3. REGRAS OPERACIONAIS</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>O resultado considerado é sempre o placar de 90 minutos.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Prorrogação e pênaltis são usados apenas para definir o classificado do mata-mata.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>A classificação e a premiação são calculadas por fase vigente.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Em caso de empate na liderança, a bolada é dividida igualmente entre os líderes.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Não existe taxa administrativa; a premiação é composta apenas pela soma das inscrições captadas.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>4. PRAZOS E RESPONSABILIDADES</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>O apostador é responsável pela conferência dos dados de identificação, do pagamento e dos palpites antes do envio.</t>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>O apostador é responsável pela conferência dos dados de identificação, pagamento e palpites antes do envio.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>A organização pode atualizar o arquivo, fechar a captação ou republicar nova versão quando houver correção oficial.</t>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>A organização pode atualizar o arquivo, fechar a captação ou publicar nova versão quando houver correção oficial.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Os confrontos seguintes dependem do chaveamento oficial e da definição dos classificados em cada fase.</t>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>A consolidação futura deve usar os arquivos oficiais e a nomenclatura oficial da FIFA.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza confrontos oficiais da fase de 32 avos
</commit_message>
<xml_diff>
--- a/public/bolao_copa2026_final_envio.xlsx
+++ b/public/bolao_copa2026_final_envio.xlsx
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="B2:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -613,7 +613,6 @@
     <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="10" t="inlineStr">
         <is>
@@ -661,7 +660,6 @@
       </c>
     </row>
     <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="B8" s="12" t="inlineStr">
         <is>
@@ -741,8 +739,6 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -818,7 +814,7 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo A</t>
+          <t>África do Sul</t>
         </is>
       </c>
       <c r="D16" s="13" t="n"/>
@@ -830,7 +826,7 @@
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo B</t>
+          <t>Canadá</t>
         </is>
       </c>
       <c r="H16" s="13" t="n"/>
@@ -852,7 +848,7 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo E</t>
+          <t>Alemanha</t>
         </is>
       </c>
       <c r="D17" s="13" t="n"/>
@@ -864,7 +860,7 @@
       <c r="F17" s="13" t="n"/>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos A/B/C/D/F</t>
+          <t>Paraguai</t>
         </is>
       </c>
       <c r="H17" s="13" t="n"/>
@@ -886,7 +882,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo F</t>
+          <t>Holanda</t>
         </is>
       </c>
       <c r="D18" s="13" t="n"/>
@@ -898,7 +894,7 @@
       <c r="F18" s="13" t="n"/>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo C</t>
+          <t>Marrocos</t>
         </is>
       </c>
       <c r="H18" s="13" t="n"/>
@@ -920,7 +916,7 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo C</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="D19" s="13" t="n"/>
@@ -932,7 +928,7 @@
       <c r="F19" s="13" t="n"/>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo F</t>
+          <t>Japão</t>
         </is>
       </c>
       <c r="H19" s="13" t="n"/>
@@ -954,7 +950,7 @@
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo I</t>
+          <t>França</t>
         </is>
       </c>
       <c r="D20" s="13" t="n"/>
@@ -966,7 +962,7 @@
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos C/D/F/G/H</t>
+          <t>Suécia</t>
         </is>
       </c>
       <c r="H20" s="13" t="n"/>
@@ -988,7 +984,7 @@
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo E</t>
+          <t>Costa do Marfim</t>
         </is>
       </c>
       <c r="D21" s="13" t="n"/>
@@ -1000,7 +996,7 @@
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo I</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="H21" s="13" t="n"/>
@@ -1022,7 +1018,7 @@
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo A</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D22" s="13" t="n"/>
@@ -1034,7 +1030,7 @@
       <c r="F22" s="13" t="n"/>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos C/E/F/H/I</t>
+          <t>Equador</t>
         </is>
       </c>
       <c r="H22" s="13" t="n"/>
@@ -1056,7 +1052,7 @@
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo L</t>
+          <t>Inglaterra</t>
         </is>
       </c>
       <c r="D23" s="13" t="n"/>
@@ -1068,7 +1064,7 @@
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos E/H/I/J/K</t>
+          <t>RD Congo</t>
         </is>
       </c>
       <c r="H23" s="13" t="n"/>
@@ -1090,7 +1086,7 @@
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo D</t>
+          <t>Bélgica</t>
         </is>
       </c>
       <c r="D24" s="13" t="n"/>
@@ -1102,7 +1098,7 @@
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos B/E/F/I/J</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="H24" s="13" t="n"/>
@@ -1124,7 +1120,7 @@
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo G</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="D25" s="13" t="n"/>
@@ -1136,7 +1132,7 @@
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos A/E/H/I/J</t>
+          <t>Bósnia</t>
         </is>
       </c>
       <c r="H25" s="13" t="n"/>
@@ -1158,7 +1154,7 @@
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo K</t>
+          <t>Espanha</t>
         </is>
       </c>
       <c r="D26" s="13" t="n"/>
@@ -1170,7 +1166,7 @@
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo L</t>
+          <t>Áustria</t>
         </is>
       </c>
       <c r="H26" s="13" t="n"/>
@@ -1192,7 +1188,7 @@
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo H</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="D27" s="13" t="n"/>
@@ -1204,7 +1200,7 @@
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo J</t>
+          <t>Croácia</t>
         </is>
       </c>
       <c r="H27" s="13" t="n"/>
@@ -1226,7 +1222,7 @@
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo B</t>
+          <t>Suíça</t>
         </is>
       </c>
       <c r="D28" s="13" t="n"/>
@@ -1238,7 +1234,7 @@
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos E/F/G/I/J</t>
+          <t>Argélia</t>
         </is>
       </c>
       <c r="H28" s="13" t="n"/>
@@ -1260,7 +1256,7 @@
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo J</t>
+          <t>Austrália</t>
         </is>
       </c>
       <c r="D29" s="13" t="n"/>
@@ -1272,7 +1268,7 @@
       <c r="F29" s="13" t="n"/>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo H</t>
+          <t>Egito</t>
         </is>
       </c>
       <c r="H29" s="13" t="n"/>
@@ -1294,7 +1290,7 @@
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo K</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="D30" s="13" t="n"/>
@@ -1306,7 +1302,7 @@
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos D/E/I/J/L</t>
+          <t>Cabo Verde</t>
         </is>
       </c>
       <c r="H30" s="13" t="n"/>
@@ -1328,7 +1324,7 @@
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo D</t>
+          <t>Colômbia</t>
         </is>
       </c>
       <c r="D31" s="13" t="n"/>
@@ -1340,7 +1336,7 @@
       <c r="F31" s="13" t="n"/>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo G</t>
+          <t>Gana</t>
         </is>
       </c>
       <c r="H31" s="13" t="n"/>
@@ -1603,12 +1599,12 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo A</t>
+          <t>África do Sul</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo B</t>
+          <t>Canadá</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -1616,9 +1612,21 @@
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr"/>
-      <c r="G2" s="1" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I2" s="13" t="n"/>
       <c r="J2" s="13" t="n"/>
       <c r="K2" s="13">
@@ -1649,12 +1657,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo E</t>
+          <t>Alemanha</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos A/B/C/D/F</t>
+          <t>Paraguai</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -1662,9 +1670,21 @@
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr"/>
-      <c r="G3" s="1" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Gillette Stadium</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I3" s="13" t="n"/>
       <c r="J3" s="13" t="n"/>
       <c r="K3" s="13">
@@ -1695,12 +1715,12 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo F</t>
+          <t>Holanda</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo C</t>
+          <t>Marrocos</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
@@ -1708,9 +1728,21 @@
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr"/>
-      <c r="G4" s="1" t="inlineStr"/>
-      <c r="H4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Estádio BBVA</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>MEX</t>
+        </is>
+      </c>
       <c r="I4" s="13" t="n"/>
       <c r="J4" s="13" t="n"/>
       <c r="K4" s="13">
@@ -1741,12 +1773,12 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo C</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo F</t>
+          <t>Japão</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -1754,9 +1786,21 @@
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr"/>
-      <c r="G5" s="1" t="inlineStr"/>
-      <c r="H5" s="1" t="inlineStr"/>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>NRG Stadium</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13" t="n"/>
       <c r="K5" s="13">
@@ -1787,12 +1831,12 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo I</t>
+          <t>França</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos C/D/F/G/H</t>
+          <t>Suécia</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -1800,9 +1844,21 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr"/>
-      <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr"/>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>MetLife Stadium</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I6" s="13" t="n"/>
       <c r="J6" s="13" t="n"/>
       <c r="K6" s="13">
@@ -1833,12 +1889,12 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo E</t>
+          <t>Costa do Marfim</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo I</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -1846,9 +1902,21 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr"/>
-      <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr"/>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I7" s="13" t="n"/>
       <c r="J7" s="13" t="n"/>
       <c r="K7" s="13">
@@ -1879,12 +1947,12 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo A</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos C/E/F/H/I</t>
+          <t>Equador</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
@@ -1892,9 +1960,21 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr"/>
-      <c r="G8" s="1" t="inlineStr"/>
-      <c r="H8" s="1" t="inlineStr"/>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Estádio Azteca</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>MEX</t>
+        </is>
+      </c>
       <c r="I8" s="13" t="n"/>
       <c r="J8" s="13" t="n"/>
       <c r="K8" s="13">
@@ -1925,12 +2005,12 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo L</t>
+          <t>Inglaterra</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos E/H/I/J/K</t>
+          <t>RD Congo</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -1938,9 +2018,21 @@
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr"/>
-      <c r="G9" s="1" t="inlineStr"/>
-      <c r="H9" s="1" t="inlineStr"/>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz Stadium</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I9" s="13" t="n"/>
       <c r="J9" s="13" t="n"/>
       <c r="K9" s="13">
@@ -1971,12 +2063,12 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo D</t>
+          <t>Bélgica</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos B/E/F/I/J</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
@@ -1984,9 +2076,21 @@
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr"/>
-      <c r="G10" s="1" t="inlineStr"/>
-      <c r="H10" s="1" t="inlineStr"/>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Lumen Field</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I10" s="13" t="n"/>
       <c r="J10" s="13" t="n"/>
       <c r="K10" s="13">
@@ -2017,12 +2121,12 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo G</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos A/E/H/I/J</t>
+          <t>Bósnia</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
@@ -2030,9 +2134,21 @@
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr"/>
-      <c r="G11" s="1" t="inlineStr"/>
-      <c r="H11" s="1" t="inlineStr"/>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Levi's Stadium</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I11" s="13" t="n"/>
       <c r="J11" s="13" t="n"/>
       <c r="K11" s="13">
@@ -2063,12 +2179,12 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo K</t>
+          <t>Espanha</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo L</t>
+          <t>Áustria</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
@@ -2076,9 +2192,21 @@
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr"/>
-      <c r="G12" s="1" t="inlineStr"/>
-      <c r="H12" s="1" t="inlineStr"/>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I12" s="13" t="n"/>
       <c r="J12" s="13" t="n"/>
       <c r="K12" s="13">
@@ -2109,12 +2237,12 @@
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo H</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo J</t>
+          <t>Croácia</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -2122,9 +2250,21 @@
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr"/>
-      <c r="G13" s="1" t="inlineStr"/>
-      <c r="H13" s="1" t="inlineStr"/>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>BMO Field</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
       <c r="I13" s="13" t="n"/>
       <c r="J13" s="13" t="n"/>
       <c r="K13" s="13">
@@ -2155,22 +2295,34 @@
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo B</t>
+          <t>Suíça</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos E/F/G/I/J</t>
+          <t>Argélia</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr"/>
-      <c r="G14" s="1" t="inlineStr"/>
-      <c r="H14" s="1" t="inlineStr"/>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>BC Place</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
       <c r="I14" s="13" t="n"/>
       <c r="J14" s="13" t="n"/>
       <c r="K14" s="13">
@@ -2201,12 +2353,12 @@
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo J</t>
+          <t>Austrália</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo H</t>
+          <t>Egito</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -2214,9 +2366,21 @@
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr"/>
-      <c r="G15" s="1" t="inlineStr"/>
-      <c r="H15" s="1" t="inlineStr"/>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I15" s="13" t="n"/>
       <c r="J15" s="13" t="n"/>
       <c r="K15" s="13">
@@ -2247,12 +2411,12 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>1º Grupo K</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>Melhor 3º colocado: Grupos D/E/I/J/L</t>
+          <t>Cabo Verde</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
@@ -2260,9 +2424,21 @@
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr"/>
-      <c r="G16" s="1" t="inlineStr"/>
-      <c r="H16" s="1" t="inlineStr"/>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Hard Rock Stadium</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I16" s="13" t="n"/>
       <c r="J16" s="13" t="n"/>
       <c r="K16" s="13">
@@ -2293,12 +2469,12 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo D</t>
+          <t>Colômbia</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>2º Grupo G</t>
+          <t>Gana</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -2306,9 +2482,21 @@
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr"/>
-      <c r="G17" s="1" t="inlineStr"/>
-      <c r="H17" s="1" t="inlineStr"/>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>Arrowhead Stadium</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
       <c r="I17" s="13" t="n"/>
       <c r="J17" s="13" t="n"/>
       <c r="K17" s="13">
@@ -2375,7 +2563,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R32 reescrito com nomenclatura oficial FIFA. Sem seleções fixas fora dos slots oficiais.</t>
+          <t>R32 atualizado com a tabela corrigida, incluindo Alemanha x Paraguai, Estados Unidos x Bósnia e demais confrontos revisados.</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2647,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Os confrontos foram mantidos como slots oficiais porque a classificação final de grupo ainda é variável.</t>
+          <t>2026-06-28 09:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alinha pontuação ao placar final com prorrogação
</commit_message>
<xml_diff>
--- a/public/bolao_copa2026_final_envio.xlsx
+++ b/public/bolao_copa2026_final_envio.xlsx
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -613,6 +613,7 @@
     <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="10" t="inlineStr">
         <is>
@@ -648,7 +649,7 @@
           <t>REGULAMENTO &amp; INSTRUÇÕES:
 1. Preencha os dados de identificação.
 2. Informe os palpites dos 32 avos.
-3. Resultados válidos: apenas 90 minutos.
+3. Resultados válidos: apenas tempo normal e a prorrogação.
 4. Prorrogação e pênaltis servem apenas para definir classificado.</t>
         </is>
       </c>
@@ -660,6 +661,7 @@
       </c>
     </row>
     <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="B8" s="12" t="inlineStr">
         <is>
@@ -739,6 +741,8 @@
         <v>50</v>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -2651,6 +2655,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -2844,7 +2849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E25"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -2853,6 +2858,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -2869,6 +2875,7 @@
       <c r="D3" s="8" t="n"/>
       <c r="E3" s="9" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="14" t="inlineStr">
         <is>
@@ -2888,6 +2895,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -2934,7 +2942,7 @@
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>3 pontos</t>
+          <t>Para pontuação, vale o placar final após o tempo normal e a prorrogação; pênaltis servem apenas para classificar.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2955,6 +2963,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="14" t="inlineStr">
         <is>
@@ -2970,7 +2979,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>O resultado considerado é sempre o placar de 90 minutos.</t>
+          <t>O resultado considerado é sempre o placar de tempo normal e a prorrogação.</t>
         </is>
       </c>
     </row>
@@ -3022,6 +3031,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="B22" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove controles extras da planilha
</commit_message>
<xml_diff>
--- a/public/bolao_copa2026_final_envio.xlsx
+++ b/public/bolao_copa2026_final_envio.xlsx
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="B2:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -613,7 +613,6 @@
     <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="10" t="inlineStr">
         <is>
@@ -621,58 +620,36 @@
         </is>
       </c>
       <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-28 / revisão FIFA</t>
-        </is>
-      </c>
+      <c r="K2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="J3" s="1" t="n"/>
-      <c r="K3" s="1" t="inlineStr">
-        <is>
-          <t>FIFA oficial</t>
-        </is>
-      </c>
+      <c r="K3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="J4" s="1" t="n"/>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-28 09:27</t>
-        </is>
-      </c>
+      <c r="K4" s="1" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="11" t="inlineStr">
         <is>
           <t>REGULAMENTO &amp; INSTRUÇÕES:
-1. Preencha os dados de identificação.
-2. Informe os palpites dos 32 avos.
-3. Resultados válidos: apenas tempo normal e a prorrogação.
-4. Prorrogação e pênaltis servem apenas para definir classificado.</t>
+1. Preencha seus dados de identificação.
+2. Informe os placares dos jogos da fase de 32 avos.
+3. Apenas os campos de identificação e placar ficam editáveis.</t>
         </is>
       </c>
       <c r="J5" s="1" t="n"/>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>48 seleções · 12 grupos · 32 avos</t>
-        </is>
-      </c>
+      <c r="K5" s="1" t="n"/>
     </row>
     <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>1. IDENTIFICAÇÃO DO APOSTADOR (Obrigatório) — Taxa: R$ 50,00 · PIX 71994793104 (Leandro Freire)</t>
-        </is>
-      </c>
-      <c r="J8" s="1" t="inlineStr">
-        <is>
-          <t>ID ÚNICO</t>
-        </is>
-      </c>
+          <t>1. IDENTIFICAÇÃO DO APOSTADOR (Obrigatório)</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="n"/>
       <c r="K8" s="1" t="n"/>
     </row>
     <row r="9">
@@ -682,11 +659,7 @@
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr"/>
-      <c r="J9" s="1" t="inlineStr">
-        <is>
-          <t>DATA/HORA DO ENVIO</t>
-        </is>
-      </c>
+      <c r="J9" s="1" t="n"/>
       <c r="K9" s="1" t="n"/>
     </row>
     <row r="10">
@@ -696,16 +669,8 @@
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr"/>
-      <c r="J10" s="1" t="inlineStr">
-        <is>
-          <t>STATUS PAGAMENTO</t>
-        </is>
-      </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="J10" s="1" t="n"/>
+      <c r="K10" s="1" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="1" t="inlineStr">
@@ -714,16 +679,8 @@
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr"/>
-      <c r="J11" s="1" t="inlineStr">
-        <is>
-          <t>CONFIRMAÇÃO PIX</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="inlineStr">
-        <is>
-          <t>Não confirmado</t>
-        </is>
-      </c>
+      <c r="J11" s="1" t="n"/>
+      <c r="K11" s="1" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="1" t="inlineStr">
@@ -732,17 +689,9 @@
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr"/>
-      <c r="J12" s="1" t="inlineStr">
-        <is>
-          <t>VALOR INSCRIÇÃO</t>
-        </is>
-      </c>
-      <c r="K12" s="13" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14"/>
+      <c r="J12" s="1" t="n"/>
+      <c r="K12" s="1" t="n"/>
+    </row>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -774,36 +723,12 @@
           <t>Seleção Visitante</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Classificado</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Decisão</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>ET M</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>ET V</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Pen M</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>Pen V</t>
-        </is>
-      </c>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="4" t="n"/>
+      <c r="L15" s="4" t="n"/>
+      <c r="M15" s="4" t="n"/>
       <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Status</t>
@@ -833,16 +758,12 @@
           <t>Canadá</t>
         </is>
       </c>
-      <c r="H16" s="13" t="n"/>
-      <c r="I16" s="13" t="n"/>
-      <c r="J16" s="13" t="n"/>
-      <c r="K16" s="13" t="n"/>
-      <c r="L16" s="13" t="n"/>
-      <c r="M16" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H16" s="1" t="n"/>
+      <c r="I16" s="1" t="n"/>
+      <c r="J16" s="1" t="n"/>
+      <c r="K16" s="1" t="n"/>
+      <c r="L16" s="1" t="n"/>
+      <c r="M16" s="1" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="1" t="inlineStr">
@@ -867,16 +788,12 @@
           <t>Paraguai</t>
         </is>
       </c>
-      <c r="H17" s="13" t="n"/>
-      <c r="I17" s="13" t="n"/>
-      <c r="J17" s="13" t="n"/>
-      <c r="K17" s="13" t="n"/>
-      <c r="L17" s="13" t="n"/>
-      <c r="M17" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H17" s="1" t="n"/>
+      <c r="I17" s="1" t="n"/>
+      <c r="J17" s="1" t="n"/>
+      <c r="K17" s="1" t="n"/>
+      <c r="L17" s="1" t="n"/>
+      <c r="M17" s="1" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="1" t="inlineStr">
@@ -901,16 +818,12 @@
           <t>Marrocos</t>
         </is>
       </c>
-      <c r="H18" s="13" t="n"/>
-      <c r="I18" s="13" t="n"/>
-      <c r="J18" s="13" t="n"/>
-      <c r="K18" s="13" t="n"/>
-      <c r="L18" s="13" t="n"/>
-      <c r="M18" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H18" s="1" t="n"/>
+      <c r="I18" s="1" t="n"/>
+      <c r="J18" s="1" t="n"/>
+      <c r="K18" s="1" t="n"/>
+      <c r="L18" s="1" t="n"/>
+      <c r="M18" s="1" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="1" t="inlineStr">
@@ -935,16 +848,12 @@
           <t>Japão</t>
         </is>
       </c>
-      <c r="H19" s="13" t="n"/>
-      <c r="I19" s="13" t="n"/>
-      <c r="J19" s="13" t="n"/>
-      <c r="K19" s="13" t="n"/>
-      <c r="L19" s="13" t="n"/>
-      <c r="M19" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H19" s="1" t="n"/>
+      <c r="I19" s="1" t="n"/>
+      <c r="J19" s="1" t="n"/>
+      <c r="K19" s="1" t="n"/>
+      <c r="L19" s="1" t="n"/>
+      <c r="M19" s="1" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="1" t="inlineStr">
@@ -969,16 +878,12 @@
           <t>Suécia</t>
         </is>
       </c>
-      <c r="H20" s="13" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
-      <c r="L20" s="13" t="n"/>
-      <c r="M20" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H20" s="1" t="n"/>
+      <c r="I20" s="1" t="n"/>
+      <c r="J20" s="1" t="n"/>
+      <c r="K20" s="1" t="n"/>
+      <c r="L20" s="1" t="n"/>
+      <c r="M20" s="1" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="1" t="inlineStr">
@@ -1003,16 +908,12 @@
           <t>Noruega</t>
         </is>
       </c>
-      <c r="H21" s="13" t="n"/>
-      <c r="I21" s="13" t="n"/>
-      <c r="J21" s="13" t="n"/>
-      <c r="K21" s="13" t="n"/>
-      <c r="L21" s="13" t="n"/>
-      <c r="M21" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H21" s="1" t="n"/>
+      <c r="I21" s="1" t="n"/>
+      <c r="J21" s="1" t="n"/>
+      <c r="K21" s="1" t="n"/>
+      <c r="L21" s="1" t="n"/>
+      <c r="M21" s="1" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="1" t="inlineStr">
@@ -1037,16 +938,12 @@
           <t>Equador</t>
         </is>
       </c>
-      <c r="H22" s="13" t="n"/>
-      <c r="I22" s="13" t="n"/>
-      <c r="J22" s="13" t="n"/>
-      <c r="K22" s="13" t="n"/>
-      <c r="L22" s="13" t="n"/>
-      <c r="M22" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H22" s="1" t="n"/>
+      <c r="I22" s="1" t="n"/>
+      <c r="J22" s="1" t="n"/>
+      <c r="K22" s="1" t="n"/>
+      <c r="L22" s="1" t="n"/>
+      <c r="M22" s="1" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="1" t="inlineStr">
@@ -1071,16 +968,12 @@
           <t>RD Congo</t>
         </is>
       </c>
-      <c r="H23" s="13" t="n"/>
-      <c r="I23" s="13" t="n"/>
-      <c r="J23" s="13" t="n"/>
-      <c r="K23" s="13" t="n"/>
-      <c r="L23" s="13" t="n"/>
-      <c r="M23" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H23" s="1" t="n"/>
+      <c r="I23" s="1" t="n"/>
+      <c r="J23" s="1" t="n"/>
+      <c r="K23" s="1" t="n"/>
+      <c r="L23" s="1" t="n"/>
+      <c r="M23" s="1" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="1" t="inlineStr">
@@ -1105,16 +998,12 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="H24" s="13" t="n"/>
-      <c r="I24" s="13" t="n"/>
-      <c r="J24" s="13" t="n"/>
-      <c r="K24" s="13" t="n"/>
-      <c r="L24" s="13" t="n"/>
-      <c r="M24" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H24" s="1" t="n"/>
+      <c r="I24" s="1" t="n"/>
+      <c r="J24" s="1" t="n"/>
+      <c r="K24" s="1" t="n"/>
+      <c r="L24" s="1" t="n"/>
+      <c r="M24" s="1" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="1" t="inlineStr">
@@ -1139,16 +1028,12 @@
           <t>Bósnia</t>
         </is>
       </c>
-      <c r="H25" s="13" t="n"/>
-      <c r="I25" s="13" t="n"/>
-      <c r="J25" s="13" t="n"/>
-      <c r="K25" s="13" t="n"/>
-      <c r="L25" s="13" t="n"/>
-      <c r="M25" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H25" s="1" t="n"/>
+      <c r="I25" s="1" t="n"/>
+      <c r="J25" s="1" t="n"/>
+      <c r="K25" s="1" t="n"/>
+      <c r="L25" s="1" t="n"/>
+      <c r="M25" s="1" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="1" t="inlineStr">
@@ -1173,16 +1058,12 @@
           <t>Áustria</t>
         </is>
       </c>
-      <c r="H26" s="13" t="n"/>
-      <c r="I26" s="13" t="n"/>
-      <c r="J26" s="13" t="n"/>
-      <c r="K26" s="13" t="n"/>
-      <c r="L26" s="13" t="n"/>
-      <c r="M26" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H26" s="1" t="n"/>
+      <c r="I26" s="1" t="n"/>
+      <c r="J26" s="1" t="n"/>
+      <c r="K26" s="1" t="n"/>
+      <c r="L26" s="1" t="n"/>
+      <c r="M26" s="1" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="1" t="inlineStr">
@@ -1207,16 +1088,12 @@
           <t>Croácia</t>
         </is>
       </c>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="n"/>
-      <c r="J27" s="13" t="n"/>
-      <c r="K27" s="13" t="n"/>
-      <c r="L27" s="13" t="n"/>
-      <c r="M27" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H27" s="1" t="n"/>
+      <c r="I27" s="1" t="n"/>
+      <c r="J27" s="1" t="n"/>
+      <c r="K27" s="1" t="n"/>
+      <c r="L27" s="1" t="n"/>
+      <c r="M27" s="1" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="1" t="inlineStr">
@@ -1241,16 +1118,12 @@
           <t>Argélia</t>
         </is>
       </c>
-      <c r="H28" s="13" t="n"/>
-      <c r="I28" s="13" t="n"/>
-      <c r="J28" s="13" t="n"/>
-      <c r="K28" s="13" t="n"/>
-      <c r="L28" s="13" t="n"/>
-      <c r="M28" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H28" s="1" t="n"/>
+      <c r="I28" s="1" t="n"/>
+      <c r="J28" s="1" t="n"/>
+      <c r="K28" s="1" t="n"/>
+      <c r="L28" s="1" t="n"/>
+      <c r="M28" s="1" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="1" t="inlineStr">
@@ -1275,16 +1148,12 @@
           <t>Egito</t>
         </is>
       </c>
-      <c r="H29" s="13" t="n"/>
-      <c r="I29" s="13" t="n"/>
-      <c r="J29" s="13" t="n"/>
-      <c r="K29" s="13" t="n"/>
-      <c r="L29" s="13" t="n"/>
-      <c r="M29" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H29" s="1" t="n"/>
+      <c r="I29" s="1" t="n"/>
+      <c r="J29" s="1" t="n"/>
+      <c r="K29" s="1" t="n"/>
+      <c r="L29" s="1" t="n"/>
+      <c r="M29" s="1" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="1" t="inlineStr">
@@ -1309,16 +1178,12 @@
           <t>Cabo Verde</t>
         </is>
       </c>
-      <c r="H30" s="13" t="n"/>
-      <c r="I30" s="13" t="n"/>
-      <c r="J30" s="13" t="n"/>
-      <c r="K30" s="13" t="n"/>
-      <c r="L30" s="13" t="n"/>
-      <c r="M30" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H30" s="1" t="n"/>
+      <c r="I30" s="1" t="n"/>
+      <c r="J30" s="1" t="n"/>
+      <c r="K30" s="1" t="n"/>
+      <c r="L30" s="1" t="n"/>
+      <c r="M30" s="1" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="1" t="inlineStr">
@@ -1343,16 +1208,12 @@
           <t>Gana</t>
         </is>
       </c>
-      <c r="H31" s="13" t="n"/>
-      <c r="I31" s="13" t="n"/>
-      <c r="J31" s="13" t="n"/>
-      <c r="K31" s="13" t="n"/>
-      <c r="L31" s="13" t="n"/>
-      <c r="M31" s="1" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
+      <c r="H31" s="1" t="n"/>
+      <c r="I31" s="1" t="n"/>
+      <c r="J31" s="1" t="n"/>
+      <c r="K31" s="1" t="n"/>
+      <c r="L31" s="1" t="n"/>
+      <c r="M31" s="1" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="8D2A"/>
@@ -1360,7 +1221,7 @@
     <mergeCell ref="B5:H6"/>
     <mergeCell ref="B2:H3"/>
   </mergeCells>
-  <dataValidations count="8">
+  <dataValidations count="2">
     <dataValidation sqref="D16:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Apenas números inteiros entre 0 e 20 são permitidos." prompt="Informe um inteiro entre 0 e 20." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>20</formula2>
@@ -1368,26 +1229,6 @@
     <dataValidation sqref="F16:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Apenas números inteiros entre 0 e 20 são permitidos." prompt="Informe um inteiro entre 0 e 20." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>20</formula2>
-    </dataValidation>
-    <dataValidation sqref="J16:J31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Apenas números inteiros entre 0 e 20 são permitidos." prompt="Informe um inteiro entre 0 e 20." type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>20</formula2>
-    </dataValidation>
-    <dataValidation sqref="K16:K31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Apenas números inteiros entre 0 e 20 são permitidos." prompt="Informe um inteiro entre 0 e 20." type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>20</formula2>
-    </dataValidation>
-    <dataValidation sqref="H16:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Mandante,Visitante"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I16:I31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Tempo normal,Prorrogação,Pênaltis"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Pendente,Confirmado"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2579,7 +2420,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nome, e-mail, WhatsApp, placares, classificado, decisão, prorrogação e pênaltis.</t>
+          <t>Nome, e-mail, WhatsApp e placares.</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2432,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cabeçalhos, fórmulas, estrutura, nomes das fases e células de cálculo.</t>
+          <t>Cabeçalhos, fórmulas e estrutura.</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2444,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Inteiros 0-20; listas suspensas para status, decisão e confirmação PIX.</t>
+          <t>Inteiros 0-20 apenas nos placares.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2456,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Havia seleções fixas e palpites bloqueados na linha de 32 avos.</t>
+          <t>Havia campos de controle/pagamento na aba principal, agora removidos.</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2468,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Apostador consegue digitar dados e palpites sem destravar fórmulas.</t>
+          <t>Apostador preenche identificação e placares sem campos extras.</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2496,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -2849,7 +2689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="B2:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -2858,7 +2698,6 @@
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -2875,7 +2714,6 @@
       <c r="D3" s="8" t="n"/>
       <c r="E3" s="9" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="14" t="inlineStr">
         <is>
@@ -2895,7 +2733,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -2963,7 +2800,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="B15" s="14" t="inlineStr">
         <is>
@@ -3031,7 +2867,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="B22" s="14" t="inlineStr">
         <is>

</xml_diff>